<commit_message>
Added notebook - Pratik
</commit_message>
<xml_diff>
--- a/fall-2022/Attendance.xlsx
+++ b/fall-2022/Attendance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VIP\Github_repos\vip-nlp\fall-2022\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B91CCCD-45E2-40DC-BB55-1A5356A83303}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC67EF81-7887-4F83-B9F6-27D4C7452F7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -437,7 +437,7 @@
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
+      <c r="K3" s="6"/>
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
       <c r="N3" s="7"/>
@@ -587,7 +587,7 @@
       <c r="H8" s="6"/>
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
+      <c r="K8" s="6"/>
       <c r="L8" s="7"/>
       <c r="M8" s="7"/>
       <c r="N8" s="7"/>

</xml_diff>